<commit_message>
Add regression and current market pricing models
</commit_message>
<xml_diff>
--- a/data/processed/apartments.xlsx
+++ b/data/processed/apartments.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J40"/>
+  <dimension ref="A1:P40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,17 +454,47 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>balcony_direction</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>directions</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>parking_count</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>storage_area_sqm</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>garden_area_sqm</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>roof_area_sqm</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>is_top_floor</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>property_type</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>notes</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>property_type</t>
         </is>
       </c>
     </row>
@@ -492,17 +522,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>35.4</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="b">
+        <v>0</v>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>garden</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>דירת גן</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>garden</t>
         </is>
       </c>
     </row>
@@ -530,17 +580,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
+          <t>South-East</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>4</v>
+      </c>
+      <c r="L3" t="n">
+        <v>32.8</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="b">
+        <v>0</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>garden</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>דירת גן</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>garden</t>
         </is>
       </c>
     </row>
@@ -568,17 +638,37 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>garden</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>דירת גן</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>garden</t>
         </is>
       </c>
     </row>
@@ -604,13 +694,33 @@
       <c r="G5" t="n">
         <v>12</v>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>South-West</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr"/>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>4</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -636,15 +746,35 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J6" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -670,15 +800,35 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
+          <t>North-West</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -704,15 +854,35 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J8" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" t="n">
+        <v>6</v>
+      </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -738,15 +908,35 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -770,13 +960,33 @@
       <c r="G10" t="n">
         <v>12</v>
       </c>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr"/>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>4</v>
+      </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -802,15 +1012,35 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
+          <t>South-East</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -836,15 +1066,35 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J12" t="n">
+        <v>2</v>
+      </c>
+      <c r="K12" t="n">
+        <v>6</v>
+      </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -868,13 +1118,33 @@
       <c r="G13" t="n">
         <v>12</v>
       </c>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>South-West</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr"/>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="b">
+        <v>0</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -898,13 +1168,33 @@
       <c r="G14" t="n">
         <v>12</v>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr"/>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
+      <c r="K14" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" t="b">
+        <v>0</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -928,13 +1218,33 @@
       <c r="G15" t="n">
         <v>12</v>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>North-West</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr"/>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
+      <c r="K15" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="b">
+        <v>0</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -960,15 +1270,35 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J16" t="n">
+        <v>2</v>
+      </c>
+      <c r="K16" t="n">
+        <v>6</v>
+      </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" t="b">
+        <v>0</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -992,13 +1322,33 @@
       <c r="G17" t="n">
         <v>12</v>
       </c>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" t="n">
+        <v>4</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="b">
+        <v>0</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1024,15 +1374,35 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
+      <c r="K18" t="n">
+        <v>4</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" t="b">
+        <v>0</v>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1058,15 +1428,35 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
+          <t>South-East</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" t="n">
+        <v>4</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="b">
+        <v>0</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1092,15 +1482,35 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J20" t="n">
+        <v>2</v>
+      </c>
+      <c r="K20" t="n">
+        <v>6</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" t="b">
+        <v>0</v>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1126,15 +1536,35 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
+          <t>South-West</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J21" t="n">
+        <v>1</v>
+      </c>
+      <c r="K21" t="n">
+        <v>4</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" t="b">
+        <v>0</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1158,13 +1588,33 @@
       <c r="G22" t="n">
         <v>12</v>
       </c>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr"/>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J22" t="n">
+        <v>1</v>
+      </c>
+      <c r="K22" t="n">
+        <v>4</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" t="b">
+        <v>0</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1190,15 +1640,35 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
+          <t>North-West</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="n">
+        <v>4</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0</v>
+      </c>
+      <c r="N23" t="b">
+        <v>0</v>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1224,15 +1694,35 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J24" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" t="n">
+        <v>6</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" t="b">
+        <v>0</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1258,15 +1748,35 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
+          <t>North-East</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="n">
+        <v>4</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" t="b">
+        <v>0</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1290,13 +1800,33 @@
       <c r="G26" t="n">
         <v>12</v>
       </c>
-      <c r="H26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr"/>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
+      <c r="K26" t="n">
+        <v>4</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" t="b">
+        <v>0</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1322,15 +1852,35 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
+          <t>South-East</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
+      <c r="K27" t="n">
+        <v>4</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" t="b">
+        <v>0</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1356,15 +1906,35 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J28" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" t="n">
+        <v>6</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" t="b">
+        <v>0</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1388,13 +1958,33 @@
       <c r="G29" t="n">
         <v>12</v>
       </c>
-      <c r="H29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>South-West</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr"/>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
+      <c r="K29" t="n">
+        <v>4</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" t="b">
+        <v>0</v>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1418,13 +2008,33 @@
       <c r="G30" t="n">
         <v>12</v>
       </c>
-      <c r="H30" t="inlineStr"/>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr"/>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
+      <c r="K30" t="n">
+        <v>4</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" t="b">
+        <v>0</v>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1450,15 +2060,35 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
+          <t>North-West</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
-      <c r="J31" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J31" t="n">
+        <v>1</v>
+      </c>
+      <c r="K31" t="n">
+        <v>4</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" t="b">
+        <v>0</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1484,15 +2114,35 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
-      <c r="J32" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J32" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" t="n">
+        <v>6</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" t="b">
+        <v>0</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1516,13 +2166,33 @@
       <c r="G33" t="n">
         <v>12</v>
       </c>
-      <c r="H33" t="inlineStr"/>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>North-East</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr"/>
-      <c r="J33" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" t="n">
+        <v>4</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" t="b">
+        <v>0</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1546,13 +2216,33 @@
       <c r="G34" t="n">
         <v>12</v>
       </c>
-      <c r="H34" t="inlineStr"/>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr"/>
-      <c r="J34" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="n">
+        <v>4</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" t="b">
+        <v>0</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1576,13 +2266,33 @@
       <c r="G35" t="n">
         <v>12</v>
       </c>
-      <c r="H35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>South-East</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr"/>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="n">
+        <v>4</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0</v>
+      </c>
+      <c r="N35" t="b">
+        <v>0</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1608,15 +2318,35 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
-      <c r="J36" t="inlineStr">
-        <is>
-          <t>regular</t>
-        </is>
-      </c>
+      <c r="J36" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" t="n">
+        <v>6</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0</v>
+      </c>
+      <c r="N36" t="b">
+        <v>0</v>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>regular</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1642,17 +2372,37 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
+          <t>South-West</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
           <t>מזרח</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr">
+      <c r="J37" t="n">
+        <v>2</v>
+      </c>
+      <c r="K37" t="n">
+        <v>8</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="N37" t="b">
+        <v>1</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>triplex</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr">
         <is>
           <t>טריפלקס</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>triplex</t>
         </is>
       </c>
     </row>
@@ -1680,17 +2430,37 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr">
+      <c r="J38" t="n">
+        <v>2</v>
+      </c>
+      <c r="K38" t="n">
+        <v>8</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
+      <c r="M38" t="n">
+        <v>78</v>
+      </c>
+      <c r="N38" t="b">
+        <v>1</v>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>triplex</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
         <is>
           <t>טריפלקס</t>
-        </is>
-      </c>
-      <c r="J38" t="inlineStr">
-        <is>
-          <t>triplex</t>
         </is>
       </c>
     </row>
@@ -1718,17 +2488,37 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
+          <t>North-West</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
           <t>מערב</t>
         </is>
       </c>
-      <c r="I39" t="inlineStr">
+      <c r="J39" t="n">
+        <v>2</v>
+      </c>
+      <c r="K39" t="n">
+        <v>8</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0</v>
+      </c>
+      <c r="M39" t="n">
+        <v>51</v>
+      </c>
+      <c r="N39" t="b">
+        <v>0</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>duplex</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr">
         <is>
           <t>דופלקס</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr">
-        <is>
-          <t>duplex</t>
         </is>
       </c>
     </row>
@@ -1754,15 +2544,35 @@
       <c r="G40" t="n">
         <v>39.6</v>
       </c>
-      <c r="H40" t="inlineStr"/>
-      <c r="I40" t="inlineStr">
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" t="n">
+        <v>8</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
+      <c r="M40" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="N40" t="b">
+        <v>0</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>duplex</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr">
         <is>
           <t>דופלקס</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr">
-        <is>
-          <t>duplex</t>
         </is>
       </c>
     </row>

</xml_diff>